<commit_message>
feat(akreditasi): xlsx tabel LED/LKPS persis bentuk PDF (judul + header bertingkat merge + baris contoh)
Sebelumnya tiap file xlsx hanya berisi blok metadata (Dokumen/Nomor/Header kolom
digabung per baris). Sekarang tiap file berisi tabel persis seperti di PDF:
judul tabel di atas (merge selebar tabel), header bertingkat dengan rowspan/
colspan, dan satu baris contoh berisi '-'.

- daftar_tabel_led_lkps.py: kembalikan hdr_rows (baris header bertingkat,
  kolom kosong artefak pymupdf digabung/dipangkas) di samping header gabungan
- generate_xlsx_tabel_led_lkps.py: tulis judul + merge grid header + baris
  contoh, Times New Roman, border tipis; skip file yang terbuka di Excel
- MD daftar tabel ikut diperbarui (judul dinormalkan)
</commit_message>
<xml_diff>
--- a/akreditasi/docs/tabel_xlsx/LED/LED-Tabel C1.12 - Pelaksanaan kebijakan, standar dan indikator terkait SDM.xlsx
+++ b/akreditasi/docs/tabel_xlsx/LED/LED-Tabel C1.12 - Pelaksanaan kebijakan, standar dan indikator terkait SDM.xlsx
@@ -26,34 +26,29 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
+      <name val="Times New Roman"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -61,22 +56,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -443,308 +450,160 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W12"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
-    <col width="26" customWidth="1" min="15" max="15"/>
-    <col width="26" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
-    <col width="26" customWidth="1" min="19" max="19"/>
-    <col width="26" customWidth="1" min="20" max="20"/>
-    <col width="26" customWidth="1" min="21" max="21"/>
-    <col width="26" customWidth="1" min="22" max="22"/>
-    <col width="26" customWidth="1" min="23" max="23"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11.45" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="16.7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="17.75" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Dokumen</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>LED — Laporan Evaluasi Diri</t>
-        </is>
-      </c>
+          <t>Tabel C1.12 Pelaksanaan kebijakan, standar dan indikator terkait SDM kompeten sebagai pelaksana SPMI</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>Nomor tabel</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>No.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>C1.12</t>
-        </is>
-      </c>
+          <t>Indikator</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>IKU/</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Sasaran/Target</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Capaian/Kinerja</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Nama tabel</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Pelaksanaan kebijakan, standar dan indikator terkait SDM kompeten sebagai pelaksana SPMI</t>
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>IKT</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>TS-2</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>TS-1</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>TS-2</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>TS-1</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>TS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Halaman cetak</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Halaman PDF</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Jumlah kolom</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Header tabel</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="M9" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="N9" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="O9" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="P9" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q9" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="R9" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="S9" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="T9" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="U9" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="V9" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="W9" s="4" t="n">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Indikator</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>IKU/ IKT</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Sasaran/Target TS-2</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>TS-1</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>TS</t>
-        </is>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P10" s="5" t="inlineStr">
-        <is>
-          <t>Capaian/Kinerja TS-2</t>
-        </is>
-      </c>
-      <c r="Q10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S10" s="5" t="inlineStr">
-        <is>
-          <t>TS-1</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V10" s="5" t="inlineStr">
-        <is>
-          <t>TS</t>
-        </is>
-      </c>
-      <c r="W10" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Catatan</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Nomor dan judul dari DAFTAR TABEL LED; posisi tabel dan header kolom dari caption bernomor di badan LED (baris header bertingkat digabung).</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="A2:A3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>